<commit_message>
feat(F-NAR-019): ATOM-AUT.ROU.001-07 La flaque de Raphaël
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.ROU.001-07.xlsx
+++ b/stories/arbres/ATOM-AUT.ROU.001-07.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut la flaque sous la gouttière. Il met une botte trop grande sur le pyjama. Une chose puis la suivante, ses bottes font ploc.</t>
+          <t>Le zinc tape le mur. Sur le zinc, un éclat de gouttière brille. Raphaël veut la flaque, maintenant, en pyjama. Il enfonce une botte : elle glisse. Il prend les deux : elles se coincent. Il refuse de foncer, met le pull, boit, enfile une botte puis l'autre. Sous le zinc, l'éclat de gouttière tient sur l'eau.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dehors, il pleut tout doux. La rue est brillante. Les toits sont tout mouillés. La gouttière chante goutte à goutte. Ploc. Ploc. La fenêtre est un peu embuée. On peut dessiner un rond sur la buée. Le zinc chante encore, tout près. Raphaël, tu entends la gouttière ? Oui, papa. Ça chante. La pluie fait sa musique. En ce moment, Raphaël ouvre les yeux. On entend encore les gouttes. Je veux la flaque. Les bottes vertes sont près du lit. Raphaël met une botte. Il est encore en pyjama. La botte est trop grande. Il s'assoit sur le tapis. Elle glisse. La flaque t'attend. D'abord les vêtements. Une chose, puis la suivante. Raphaël retire la botte. Il touche la buée du doigt. Le doigt laisse un petit trait. On se lève ? Oui. Raphaël se lève. Ses pieds touchent le tapis. Le pull, maintenant.</t>
+          <t>Le zinc de la gouttière tape le mur. L'air sent la pluie, un peu froid. La vitre est embuée, tiède sous le doigt. Sur le zinc, un éclat de gouttière brille. Il est tout petit, papa. C'est un éclat de gouttière. Tu entends le zinc, Raphaël ? Oui, maman. Le zinc chante, mince, contre le mur. Un rond d'eau attend sous le zinc. Ma flaque ! En ce moment, Raphaël saute du lit. Le pyjama bleu tombe sur ses genoux. Les bottes vertes attendent près du tapis. Je mets les bottes, maintenant ! Il enfonce un pied dans une botte. La botte est trop grande, trop lâche. Elle glisse, tape le tapis. Elle glisse, papa ! Tes pieds sont dans le pyjama. Il prend l'autre botte, d'un coup. Les deux bottes se coincent. Ça ne veut pas ! Raphaël tire vers la porte. Une botte reste collée au tapis. Il trébuche, assis sur le pyjama. Oh. Le sourire de Raphaël disparaît. L'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu regardes tes pieds, Raphaël ? Le pull attend sur la chaise.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Dehors, il pleut tout doux. La rue est brillante. Les toits sont tout mouillés. La gouttière chante goutte à goutte. Ploc. Ploc. La fenêtre est un peu embuée. On peut dessiner un rond sur la buée. Le zinc chante encore, tout près. Raphaël, tu entends la gouttière ? Oui, papa. Ça chante. La pluie fait sa musique. En ce moment, Raphaël ouvre les yeux. On entend encore les gouttes. Je veux la flaque. Les bottes vertes sont près du lit. Raphaël met une botte. Il est encore en pyjama. La botte est trop grande. Il s'assoit sur le tapis. Elle glisse. La flaque t'attend. D'abord les vêtements. Une chose, puis la suivante. Raphaël retire la botte. Il touche la buée du doigt. Le doigt laisse un petit trait. On se lève ? Oui. Raphaël se lève. Ses pieds touchent le tapis. Le pull, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le zinc de la gouttière tape le mur. L'air sent la pluie, un peu froid. La vitre est embuée, tiède sous le doigt. Sur le zinc, un &lt;emphasis level="moderate"&gt;éclat de gouttière&lt;/emphasis&gt; brille. Il est tout petit, papa. C'est un éclat de gouttière. Tu entends le zinc, Raphaël ? Oui, maman. Le zinc chante, mince, contre le mur. Un rond d'eau attend sous le zinc. Ma flaque ! En ce moment, Raphaël saute du lit. Le pyjama bleu tombe sur ses genoux. Les bottes vertes attendent près du tapis. Je mets les bottes, maintenant ! Il enfonce un pied dans une botte. La botte est trop grande, trop lâche. Elle glisse, tape le tapis. Elle glisse, papa ! Tes pieds sont dans le pyjama. Il prend l'autre botte, d'un coup. Les deux bottes se coincent. Ça ne veut pas ! Raphaël tire vers la porte. Une botte reste collée au tapis. Il trébuche, assis sur le pyjama. Oh. Le sourire de Raphaël disparaît. L'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu regardes tes pieds, Raphaël ? Le pull attend sur la chaise.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le soleil entre. Boris ouvre les yeux. Le drap est chaud. Papa dit : c'est le matin. &lt;emphasis&gt;une&lt;/emphasis&gt; étape après l'autre. D'abord, Boris se lève. Ses pieds touchent le tapis. Le tapis est doux. Ensuite, Boris s'habille. Il met le pull vert. Il met le pantalon. Maman dit : maintenant, le déjeuner. Boris s'assoit à table. Il mange du pain. Il boit du lait tiède. Papa dit : ensuite, le sac. Boris met la gourde dans le sac. Boris met le doudou dans le sac. Chaque étape est finie. Boris est prêt. Papa dit : une étape après l'autre. C'est plus calme.&lt;/slow&gt; [pause]</t>
+          <t>Le zinc de la gouttière tape le mur. L'air sent la pluie, un peu froid. La vitre est embuée, tiède sous le doigt. Sur le zinc, un &lt;emphasis&gt;éclat de gouttière&lt;/emphasis&gt; brille. Il est tout petit, papa. C'est un éclat de gouttière. Tu entends le zinc, Raphaël ? Oui, maman. Le zinc chante, mince, contre le mur. Un rond d'eau attend sous le zinc. Ma flaque ! En ce moment, Raphaël saute du lit. Le pyjama bleu tombe sur ses genoux. Les bottes vertes attendent près du tapis. Je mets les bottes, maintenant ! Il enfonce un pied dans une botte. La botte est trop grande, trop lâche. Elle glisse, tape le tapis. Elle glisse, papa ! Tes pieds sont dans le pyjama. Il prend l'autre botte, d'un coup. Les deux bottes se coincent. Ça ne veut pas ! Raphaël tire vers la porte. Une botte reste collée au tapis. Il trébuche, assis sur le pyjama. Oh. Le sourire de Raphaël disparaît. L'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu regardes tes pieds, Raphaël ? Le pull attend sur la chaise. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de gouttière</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,44 +1319,47 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_flaque_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Dehors, il pleut tout doux.
-narrateur|La rue est brillante.
-narrateur|Les toits sont tout mouillés.
-narrateur|La gouttière chante goutte à goutte.
-narrateur|Ploc.
-narrateur|Ploc.
-narrateur|La fenêtre est un peu embuée.
-narrateur|On peut dessiner un rond sur la buée.
-narrateur|Le zinc chante encore, tout près.
-papa|Raphaël, tu entends la gouttière ?
-enfant-m|Oui, papa.
-enfant-m|Ça chante.
-maman|La pluie fait sa musique.
-narrateur|En ce moment, Raphaël ouvre les yeux.
-narrateur|On entend encore les gouttes.
-enfant-m|Je veux la flaque.
-narrateur|Les bottes vertes sont près du lit.
-narrateur|Raphaël met une botte.
-narrateur|Il est encore en pyjama.
-narrateur|La botte est trop grande.
-narrateur|Il s'assoit sur le tapis.
-enfant-m|Elle glisse.
-papa|La flaque t'attend.
-maman|D'abord les vêtements.
-maman|Une chose, puis la suivante.
-narrateur|Raphaël retire la botte.
-narrateur|Il touche la buée du doigt.
-narrateur|Le doigt laisse un petit trait.
-papa|On se lève ?
-enfant-m|Oui.
-narrateur|Raphaël se lève.
-narrateur|Ses pieds touchent le tapis.
-papa|Le pull, maintenant.</t>
+          <t>narrateur|Le zinc de la gouttière tape le mur.
+narrateur|L'air sent la pluie, un peu froid.
+narrateur|La vitre est embuée, tiède sous le doigt.
+narrateur|Sur le zinc, un éclat de gouttière brille.
+enfant-m|Il est tout petit, papa.
+papa|C'est un éclat de gouttière.
+maman|Tu entends le zinc, Raphaël ?
+enfant-m|Oui, maman.
+narrateur|Le zinc chante, mince, contre le mur.
+narrateur|Un rond d'eau attend sous le zinc.
+enfant-m|Ma flaque !
+narrateur|En ce moment, Raphaël saute du lit.
+narrateur|Le pyjama bleu tombe sur ses genoux.
+narrateur|Les bottes vertes attendent près du tapis.
+enfant-m|Je mets les bottes, maintenant !
+narrateur|Il enfonce un pied dans une botte.
+narrateur|La botte est trop grande, trop lâche.
+narrateur|Elle glisse, tape le tapis.
+enfant-m|Elle glisse, papa !
+papa|Tes pieds sont dans le pyjama.
+narrateur|Il prend l'autre botte, d'un coup.
+narrateur|Les deux bottes se coincent.
+enfant-m|Ça ne veut pas !
+narrateur|Raphaël tire vers la porte.
+narrateur|Une botte reste collée au tapis.
+narrateur|Il trébuche, assis sur le pyjama.
+enfant-m|Oh.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|L'envie et l'inquiétude se bousculent.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu regardes tes pieds, Raphaël ?
+maman|Le pull attend sur la chaise.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1388,27 +1391,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël veut la flaque. Comment se prépare-t-il ?</t>
+          <t>Raphaël veut la flaque. Que met-il avant les bottes ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël veut la flaque. Comment se prépare-t-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Raphaël veut la flaque. Que met-il avant les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Boris se prépare. Comment avance-t-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Raphaël veut la flaque. Que met-il avant les &lt;emphasis&gt;bottes&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>une chose</t>
+          <t>le pull</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>une chose | puis l'autre | d'abord | doucement | une chose puis l'autre | puis la suivante</t>
+          <t>le pull | pull | le pull bleu | les vêtements | d'abord le pull | avant les bottes | le pyjama non</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1423,7 +1426,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il fait une chose, puis la suivante. Comment se prépare Raphaël ?</t>
+          <t>Le pull attend. Que met Raphaël avant les bottes ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1461,7 +1464,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1469,10 +1472,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1487,34 +1490,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>bottes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1523,13 +1530,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1539,13 +1546,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_pull_avant_les_bottes; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Raphaël veut la flaque.
-narrateur|Comment se prépare-t-il ?</t>
+narrateur|Que met-il avant les bottes ?</t>
         </is>
       </c>
     </row>
@@ -1572,17 +1579,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le pull bleu est sur la chaise. Raphaël enfile le pull. Le pull est un peu rêche. C'est fait. Ensuite, le bol. Raphaël va à la cuisine. Le carrelage est froid. Ça sent le lait. Tu veux le bol vert ? Oui, le vert. Il s'assoit. Il boit une gorgée. Les bottes, après le bol. Pour la flaque. Merci, Raphaël.</t>
+          <t>Raphaël refuse de forcer l'autre botte. Il retire le pied, sans tirer. La botte verte reste sur le tapis. Je mets le pull. Le pull bleu est sur la chaise. Il enfile le pull, un peu rêche. C'est fait. Tu viens au bol ? Raphaël va vers la cuisine. Le carrelage est froid sous les pieds. Ça sent le lait, tiède. Tu veux le bol vert ? Oui, le vert. Il s'assoit, près de la table. Une gorgée, puis une autre. Les bottes, maintenant ! Il saisit les deux bottes ensemble. Elles se coincent, retombent. Oh. Ses épaules tombent un peu. Il ne reprend pas trop vite. Il écoute le zinc, un instant. Sur la vitre, l'éclat de gouttière brille. Il est là. Raphaël refuse de foncer. Il glisse un pied, puis l'autre. Les bottes tiennent, fermes. Merci, Raphaël. Elles restent. On peut ouvrir ? Oui, pour la flaque.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le pull bleu est sur la chaise. Raphaël enfile le pull. Le pull est un peu rêche. C'est fait. Ensuite, le bol. Raphaël va à la cuisine. Le carrelage est froid. Ça sent le lait. Tu veux le bol vert ? Oui, le vert. Il s'assoit. Il boit une gorgée. Les bottes, après le bol. Pour la flaque. Merci, Raphaël.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël refuse de forcer l'autre botte. Il retire le pied, sans tirer. La botte verte reste sur le tapis. Je mets le pull. Le pull bleu est sur la chaise. Il enfile le pull, un peu rêche. C'est fait. Tu viens au bol ? Raphaël va vers la cuisine. Le carrelage est froid sous les pieds. Ça sent le lait, tiède. Tu veux le bol vert ? Oui, le vert. Il s'assoit, près de la table. Une gorgée, puis une autre. Les bottes, maintenant ! Il saisit les deux bottes ensemble. Elles se coincent, retombent. Oh. Ses épaules tombent un peu. Il ne reprend pas trop vite. Il écoute le zinc, un instant. Sur la vitre, l'&lt;emphasis level="moderate"&gt;éclat de gouttière&lt;/emphasis&gt; brille. Il est là. Raphaël refuse de foncer. Il glisse un pied, puis l'autre. Les bottes tiennent, fermes. Merci, Raphaël. Elles restent. On peut ouvrir ? Oui, pour la flaque.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Boris a fait l'étape dite. Se lever. S'habiller. Déje&lt;emphasis&gt;une&lt;/emphasis&gt;r. Le sac. Une étape après l'autre.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël refuse de forcer l'autre botte. Il retire le pied, sans tirer. La botte verte reste sur le tapis. Je mets le pull. Le pull bleu est sur la chaise. Il enfile le pull, un peu rêche. C'est fait. Tu viens au bol ? Raphaël va vers la cuisine. Le carrelage est froid sous les pieds. Ça sent le lait, tiède. Tu veux le bol vert ? Oui, le vert. Il s'assoit, près de la table. Une gorgée, puis une autre. Les bottes, maintenant ! Il saisit les deux bottes ensemble. Elles se coincent, retombent. Oh. Ses épaules tombent un peu. Il ne reprend pas trop vite. Il écoute le zinc, un instant. Sur la vitre, l'&lt;emphasis&gt;éclat de gouttière&lt;/emphasis&gt; brille. Il est là. Raphaël refuse de foncer. Il glisse un pied, puis l'autre. Les bottes tiennent, fermes. Merci, Raphaël. Elles restent. On peut ouvrir ? Oui, pour la flaque. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1629,7 +1636,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1637,10 +1644,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1663,30 +1670,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de gouttière</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1695,10 +1702,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1707,30 +1714,51 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_met_le_pull_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Le pull bleu est sur la chaise.
-narrateur|Raphaël enfile le pull.
-narrateur|Le pull est un peu rêche.
+          <t>narrateur|Raphaël refuse de forcer l'autre botte.
+narrateur|Il retire le pied, sans tirer.
+narrateur|La botte verte reste sur le tapis.
+enfant-m|Je mets le pull.
+narrateur|Le pull bleu est sur la chaise.
+narrateur|Il enfile le pull, un peu rêche.
 enfant-m|C'est fait.
-maman|Ensuite, le bol.
-narrateur|Raphaël va à la cuisine.
-narrateur|Le carrelage est froid.
-narrateur|Ça sent le lait.
+maman|Tu viens au bol ?
+narrateur|Raphaël va vers la cuisine.
+narrateur|Le carrelage est froid sous les pieds.
+narrateur|Ça sent le lait, tiède.
 papa|Tu veux le bol vert ?
 enfant-m|Oui, le vert.
-narrateur|Il s'assoit.
-narrateur|Il boit une gorgée.
-maman|Les bottes, après le bol.
-enfant-m|Pour la flaque.
-papa|Merci, Raphaël.</t>
+narrateur|Il s'assoit, près de la table.
+narrateur|Une gorgée, puis une autre.
+enfant-m|Les bottes, maintenant !
+narrateur|Il saisit les deux bottes ensemble.
+narrateur|Elles se coincent, retombent.
+enfant-m|Oh.
+narrateur|Ses épaules tombent un peu.
+narrateur|Il ne reprend pas trop vite.
+narrateur|Il écoute le zinc, un instant.
+narrateur|Sur la vitre, l'éclat de gouttière brille.
+enfant-m|Il est là.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il glisse un pied, puis l'autre.
+narrateur|Les bottes tiennent, fermes.
+papa|Merci, Raphaël.
+enfant-m|Elles restent.
+maman|On peut ouvrir ?
+enfant-m|Oui, pour la flaque.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pull,bol</t>
         </is>
       </c>
     </row>
@@ -1757,17 +1785,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ensuite, les bottes. Raphaël enfile une botte. Puis l'autre. Elles ne glissent plus. Le bon pied ? Oui. Maman ouvre la porte. L'air sent la pluie. La gouttière chante encore. Sous le zinc, une flaque ronde attend. Elle est là. Un pied, puis l'autre. Raphaël pose une botte dans l'eau. Ça fait ploc. Puis l'autre botte. Ça fait ploc encore. C'est froid. Oui, tout doux. Un cercle d'eau s'ouvre. On en fait un autre ? Oui. Raphaël saute un tout petit peu. L'eau saute aussi, toute claire. Un rond de buée reste à la fenêtre. La rue brille encore, tout loin. Tes pieds sont au chaud ? Oui, dans les bottes. Une goutte tombe encore du zinc. Elle fait un nouveau cercle. Tu as attendu tes vêtements ? Oui, une chose, puis l'autre.</t>
+          <t>J'ouvre la porte. Maman pousse la porte, un peu. L'air sent la pluie, frais. Le zinc chante, mince, au-dessus. Sous le zinc, une flaque ronde attend. Elle est là ! Tu poses un pied ? Les deux, maintenant ! Raphaël recule d'un pas. Il refuse de foncer. Une botte entre dans l'eau. Ça fait ploc. Puis l'autre botte. Ça fait ploc, plus large. C'est froid. Tes pieds sont au chaud ? Oui, dans les bottes. Un cercle d'eau s'ouvre. On en fait un autre ? Oui. Raphaël saute un tout petit peu. L'eau saute aussi, claire. Un rond de buée reste à la vitre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ensuite, les bottes. Raphaël enfile une botte. Puis l'autre. Elles ne glissent plus. Le bon pied ? Oui. Maman ouvre la porte. L'air sent la pluie. La gouttière chante encore. Sous le zinc, une flaque ronde attend. Elle est là. Un pied, puis l'autre. Raphaël pose une botte dans l'eau. Ça fait ploc. Puis l'autre botte. Ça fait ploc encore. C'est froid. Oui, tout doux. Un cercle d'eau s'ouvre. On en fait un autre ? Oui. Raphaël saute un tout petit peu. L'eau saute aussi, toute claire. Un rond de buée reste à la fenêtre. La rue brille encore, tout loin. Tes pieds sont au chaud ? Oui, dans les bottes. Une goutte tombe encore du zinc. Elle fait un nouveau cercle. Tu as attendu tes vêtements ? Oui, une chose, puis l'autre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'ouvre la porte. Maman pousse la porte, un peu. L'air sent la pluie, frais. Le zinc chante, mince, au-dessus. Sous le zinc, une &lt;emphasis level="moderate"&gt;flaque&lt;/emphasis&gt; ronde attend. Elle est là ! Tu poses un pied ? Les deux, maintenant ! Raphaël recule d'un pas. Il refuse de foncer. Une botte entre dans l'eau. Ça fait ploc. Puis l'autre botte. Ça fait ploc, plus large. C'est froid. Tes pieds sont au chaud ? Oui, dans les bottes. Un cercle d'eau s'ouvre. On en fait un autre ? Oui. Raphaël saute un tout petit peu. L'eau saute aussi, claire. Un rond de buée reste à la vitre.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Boris met les chaussures. Maman ouvre la porte. L'air sent le matin.&lt;/slow&gt; [pause]</t>
+          <t>J'ouvre la porte. Maman pousse la porte, un peu. L'air sent la pluie, frais. Le zinc chante, mince, au-dessus. Sous le zinc, une &lt;emphasis&gt;flaque&lt;/emphasis&gt; ronde attend. Elle est là ! Tu poses un pied ? Les deux, maintenant ! Raphaël recule d'un pas. Il refuse de foncer. Une botte entre dans l'eau. Ça fait ploc. Puis l'autre botte. Ça fait ploc, plus large. C'est froid. Tes pieds sont au chaud ? Oui, dans les bottes. Un cercle d'eau s'ouvre. On en fait un autre ? Oui. Raphaël saute un tout petit peu. L'eau saute aussi, claire. Un rond de buée reste à la vitre. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1814,7 +1842,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1822,10 +1850,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1846,28 +1874,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>flaque</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1876,10 +1908,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1888,47 +1920,43 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_sauter_des_deux_pieds; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|Ensuite, les bottes.
-narrateur|Raphaël enfile une botte.
-narrateur|Puis l'autre.
-narrateur|Elles ne glissent plus.
-papa|Le bon pied ?
-enfant-m|Oui.
-narrateur|Maman ouvre la porte.
-narrateur|L'air sent la pluie.
-narrateur|La gouttière chante encore.
+          <t>maman|J'ouvre la porte.
+narrateur|Maman pousse la porte, un peu.
+narrateur|L'air sent la pluie, frais.
+narrateur|Le zinc chante, mince, au-dessus.
 narrateur|Sous le zinc, une flaque ronde attend.
-enfant-m|Elle est là.
-papa|Un pied, puis l'autre.
-narrateur|Raphaël pose une botte dans l'eau.
+enfant-m|Elle est là !
+papa|Tu poses un pied ?
+enfant-m|Les deux, maintenant !
+narrateur|Raphaël recule d'un pas.
+narrateur|Il refuse de foncer.
+narrateur|Une botte entre dans l'eau.
 narrateur|Ça fait ploc.
 narrateur|Puis l'autre botte.
-narrateur|Ça fait ploc encore.
+narrateur|Ça fait ploc, plus large.
 enfant-m|C'est froid.
-maman|Oui, tout doux.
+maman|Tes pieds sont au chaud ?
+enfant-m|Oui, dans les bottes.
 narrateur|Un cercle d'eau s'ouvre.
 papa|On en fait un autre ?
 enfant-m|Oui.
 narrateur|Raphaël saute un tout petit peu.
-narrateur|L'eau saute aussi, toute claire.
-narrateur|Un rond de buée reste à la fenêtre.
-narrateur|La rue brille encore, tout loin.
-maman|Tes pieds sont au chaud ?
-enfant-m|Oui, dans les bottes.
-narrateur|Une goutte tombe encore du zinc.
-narrateur|Elle fait un nouveau cercle.
-papa|Tu as attendu tes vêtements ?
-enfant-m|Oui, une chose, puis l'autre.</t>
+narrateur|L'eau saute aussi, claire.
+narrateur|Un rond de buée reste à la vitre.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>porte</t>
+          <t>porte,flaque</t>
         </is>
       </c>
     </row>
@@ -1955,17 +1983,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Mes bottes ont chanté. Une chose, puis la suivante. La gouttière et toi, ensemble. Le zinc chante encore, tout près. Bravo, Raphaël. La flaque ronde tremble encore sous les bottes.</t>
+          <t>Ils restent dans la flaque ronde. L'eau touche le cuir des bottes. Ma flaque chante. Oui, près de toi. Sur l'eau, un éclat de gouttière brille. Comme sur le zinc, papa ! Tu le vois, toi ? Oui, sur l'eau. Raphaël recule le pied, sans se presser. Le cuir repose dans le cercle. On le sent, maman. Tu le sens sur tes joues ? Oui, il est frais. Le zinc repose contre le mur. L'éclat de gouttière tient sur l'eau.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Mes bottes ont chanté. Une chose, puis la suivante. La gouttière et toi, ensemble. Le zinc chante encore, tout près. Bravo, Raphaël. La flaque ronde tremble encore sous les bottes.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent dans la flaque ronde. L'eau touche le cuir des bottes. Ma flaque chante. Oui, près de toi. Sur l'eau, un &lt;emphasis level="moderate"&gt;éclat de gouttière&lt;/emphasis&gt; brille. Comme sur le zinc, papa ! Tu le vois, toi ? Oui, sur l'eau. Raphaël recule le pied, sans se presser. Le cuir repose dans le cercle. On le sent, maman. Tu le sens sur tes joues ? Oui, il est frais. Le zinc repose contre le mur. L'éclat de gouttière tient sur l'eau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent dans la flaque ronde. L'eau touche le cuir des bottes. Ma flaque chante. Oui, près de toi. Sur l'eau, un &lt;emphasis&gt;éclat de gouttière&lt;/emphasis&gt; brille. Comme sur le zinc, papa ! Tu le vois, toi ? Oui, sur l'eau. Raphaël recule le pied, sans se presser. Le cuir repose dans le cercle. On le sent, maman. Tu le sens sur tes joues ? Oui, il est frais. Le zinc repose contre le mur. L'éclat de gouttière tient sur l'eau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2012,18 +2040,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2032,12 +2060,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2046,17 +2074,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de gouttière</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2065,11 +2097,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2078,29 +2110,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_l_eau; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Mes bottes ont chanté.
-papa|Une chose, puis la suivante.
-maman|La gouttière et toi, ensemble.
-narrateur|Le zinc chante encore, tout près.
-papa|Bravo, Raphaël.
-narrateur|La flaque ronde tremble encore sous les bottes.</t>
+          <t>narrateur|Ils restent dans la flaque ronde.
+narrateur|L'eau touche le cuir des bottes.
+enfant-m|Ma flaque chante.
+maman|Oui, près de toi.
+narrateur|Sur l'eau, un éclat de gouttière brille.
+enfant-m|Comme sur le zinc, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur l'eau.
+narrateur|Raphaël recule le pied, sans se presser.
+narrateur|Le cuir repose dans le cercle.
+enfant-m|On le sent, maman.
+maman|Tu le sens sur tes joues ?
+enfant-m|Oui, il est frais.
+narrateur|Le zinc repose contre le mur.
+narrateur|L'éclat de gouttière tient sur l'eau.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>zinc,eau</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2213,6 +2263,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>